<commit_message>
[IMP][BE] carry forward previous-year benefits into calculation
Accepts an optional previous-benefits file on the employee-benefits
endpoint, merges its balances into the current calculation via
compute_carry_forward, and reports duplicate employee ids as a new
exception category.
</commit_message>
<xml_diff>
--- a/backend/data/Employee_Benefit_Template.xlsx
+++ b/backend/data/Employee_Benefit_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Serichai\program\Employee_Benefit_Calculation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Serichai\source_code\serichai-web-portal\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFB31C3-8A38-446F-99AD-E618B28479CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F23528-944B-42CB-9505-5203053CA785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{7750C647-E942-4770-A723-F9258ACF3C9B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>ลำดับ</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>อายุ (ปี/เดือน)</t>
+  </si>
+  <si>
+    <t>รหัสพนักงาน</t>
   </si>
 </sst>
 </file>
@@ -673,41 +676,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A29FD900-7F8B-4D90-9FA5-D49F30819027}">
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="8.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" style="6"/>
-    <col min="4" max="4" width="14.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1796875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.81640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.1796875" style="6" customWidth="1"/>
-    <col min="19" max="19" width="8.7265625" style="6"/>
-    <col min="20" max="20" width="10.54296875" style="6" customWidth="1"/>
-    <col min="21" max="16384" width="8.7265625" style="6"/>
+    <col min="1" max="2" width="8.7265625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" style="6"/>
+    <col min="5" max="5" width="14.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.90625" style="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.7265625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="10.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.1796875" style="6" customWidth="1"/>
+    <col min="20" max="20" width="8.7265625" style="6"/>
+    <col min="21" max="21" width="10.54296875" style="6" customWidth="1"/>
+    <col min="22" max="16384" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="20">
+    <row r="1" spans="1:25" ht="20">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="2"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
+      <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
@@ -717,55 +720,57 @@
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
       <c r="P1" s="4"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="3"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="5"/>
       <c r="T1" s="3"/>
       <c r="U1" s="3"/>
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
       <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
     </row>
-    <row r="2" spans="1:24" ht="20">
+    <row r="2" spans="1:25" ht="20">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="3"/>
-      <c r="F2" s="7" t="s">
+      <c r="E2" s="3"/>
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="8">
+      <c r="H2" s="8">
         <v>243983</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="5"/>
+      <c r="J2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="9">
+      <c r="K2" s="9">
         <v>0.03</v>
       </c>
-      <c r="K2" s="4"/>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="4"/>
+      <c r="M2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="11">
+      <c r="N2" s="11">
         <v>60</v>
       </c>
-      <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="3"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="5"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
     </row>
-    <row r="3" spans="1:24" ht="24.5" customHeight="1">
+    <row r="3" spans="1:25" ht="24.5" customHeight="1">
       <c r="A3" s="13" t="s">
         <v>9</v>
       </c>
@@ -775,10 +780,10 @@
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="13"/>
+      <c r="I3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="14"/>
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
@@ -787,92 +792,96 @@
       <c r="O3" s="14"/>
       <c r="P3" s="14"/>
       <c r="Q3" s="14"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="3"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="5"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
     </row>
-    <row r="4" spans="1:24" ht="104">
+    <row r="4" spans="1:25" ht="104">
       <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="L4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="N4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="Q4" s="12" t="s">
+      <c r="R4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="T4" s="12" t="s">
+      <c r="U4" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="V4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="W4" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="W4" s="12" t="s">
+      <c r="X4" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="12" t="s">
+      <c r="Y4" s="12" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="H3:Q3"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:R3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>